<commit_message>
Changes working on week 10 homework
</commit_message>
<xml_diff>
--- a/modules/wk_10_image_analysis/DataWesternBlot.xlsx
+++ b/modules/wk_10_image_analysis/DataWesternBlot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmark\Documents\GitHub\CM515-2026\modules\wk_10_image_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1E765E-77A0-4265-80A7-4FF5FCA4EEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FCB213-BEAD-4EE5-9F85-42CB23F80B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E1EB0AB2-9595-4877-B954-BD961B5A8BE3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t>Control</t>
   </si>
@@ -209,11 +209,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$24:$B$24</c15:sqref>
+                    <c15:sqref>Sheet1!$A$25:$B$25</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$24</c:f>
+              <c:f>Sheet1!$B$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -260,11 +260,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$25:$B$25</c15:sqref>
+                    <c15:sqref>Sheet1!$A$26:$B$26</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$25</c:f>
+              <c:f>Sheet1!$B$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -311,11 +311,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$26:$B$26</c15:sqref>
+                    <c15:sqref>Sheet1!$A$27:$B$27</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$26</c:f>
+              <c:f>Sheet1!$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -362,11 +362,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$27:$B$27</c15:sqref>
+                    <c15:sqref>Sheet1!$A$28:$B$28</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$27</c:f>
+              <c:f>Sheet1!$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -413,11 +413,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$28:$B$28</c15:sqref>
+                    <c15:sqref>Sheet1!$A$29:$B$29</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$28</c:f>
+              <c:f>Sheet1!$B$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -464,11 +464,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$29:$B$29</c15:sqref>
+                    <c15:sqref>Sheet1!$A$30:$B$30</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$30</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -517,11 +517,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$30:$B$30</c15:sqref>
+                    <c15:sqref>Sheet1!$A$31:$B$31</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$30</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -570,11 +570,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$A$31:$B$31</c15:sqref>
+                    <c15:sqref>Sheet1!$A$32:$B$32</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet1!$B$31</c:f>
+              <c:f>Sheet1!$B$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -821,7 +821,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Unnormalized</a:t>
+              <a:t>Western</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Blot 1 (Not Normalized)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1486,6 +1490,910 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Western Blot</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> 1 (Not Normalized)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Area Under Curve</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>14733.083000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11511.912</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12757.083000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11586.376</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2838.3049999999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9836.7900000000009</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7504.0829999999996</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6966.0829999999996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2DD0-45A9-945D-256566FBAD0D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1432551007"/>
+        <c:axId val="1432562527"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1432551007"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Lane</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1432562527"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1432562527"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Area Under</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Curve</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1432551007"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Western Blot 1 (Normalized to Loading Control)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Area Under Curve</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$25:$A$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$25:$B$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1.7528523099674547</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.94320636737988583</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.1303446248329347</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.7467449556875454</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.18368573518366146</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.1990468854771807</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.45257692787858717</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.48282565391391857</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-638E-473D-B944-A8C7667CE66C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1432528927"/>
+        <c:axId val="1432523167"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1432528927"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Lane</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1432523167"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1432523167"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Area Under Curve</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1432528927"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1566,6 +2474,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -2070,6 +3058,1012 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2578,13 +4572,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>121920</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>110490</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>60960</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>44</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2612,16 +4606,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:rowOff>125730</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>411480</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:rowOff>125730</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2641,6 +4635,78 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>26670</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>26670</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85F1FDA1-5500-28B2-5E17-0802B631BDF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>396240</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>140970</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>140970</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C64A6C2-7DAE-B109-5949-D0F00141A450}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2966,7 +5032,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD48B5FD-D602-42EE-B7E3-AB197C57FF11}">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -3116,73 +5182,81 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>1</v>
-      </c>
-      <c r="B24">
-        <f>B2/B14</f>
-        <v>1.7528523099674547</v>
+      <c r="A24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25">
-        <f t="shared" ref="B25:B31" si="0">B3/B15</f>
-        <v>0.94320636737988583</v>
+        <f>B2/B14</f>
+        <v>1.7528523099674547</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B26">
-        <f t="shared" si="0"/>
-        <v>1.1303446248329347</v>
+        <f t="shared" ref="B26:B32" si="0">B3/B15</f>
+        <v>0.94320636737988583</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>0.7467449556875454</v>
+        <v>1.1303446248329347</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>0.18368573518366146</v>
+        <v>0.7467449556875454</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>1.1990468854771807</v>
+        <v>0.18368573518366146</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>0.45257692787858717</v>
+        <v>1.1990468854771807</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
+        <v>7</v>
+      </c>
+      <c r="B31">
+        <f t="shared" si="0"/>
+        <v>0.45257692787858717</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32">
         <v>8</v>
       </c>
-      <c r="B31">
+      <c r="B32">
         <f t="shared" si="0"/>
         <v>0.48282565391391857</v>
       </c>

</xml_diff>